<commit_message>
Add per-location Excel menus from PDF for all three locations
- Parse Shilpa Enterprise menu PDF into 46 items with prices/units
- Generate Gt world mall.xlsx, Magadi road.xlsx, Subbanna garden.xlsx
- Auto-import bundled location files on first launch (per-location stock)
- Add scripts/generate_location_menus.py to regenerate from source data

Co-authored-by: muneeswari1604 <muneeswari1604@gmail.com>
</commit_message>
<xml_diff>
--- a/assets/templates/locations/Gt world mall.xlsx
+++ b/assets/templates/locations/Gt world mall.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,66 +476,78 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>BEVARGES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BBQ Seasoning</t>
+          <t>water 1/2 liter</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BBQ Seasoning</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BEVARGES</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>pc</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>BEVARGES</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Big Buckets</t>
+          <t>cool drinks glass</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>cool drinks</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BEVARGES</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>24</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -547,27 +559,31 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>BEVARGES</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Burger Bun With Sesame</t>
+          <t>pepsi 300 ml</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Burger Bun With Sesame</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>pepsi</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BEVARGES</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>1</t>
@@ -576,7 +592,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>24</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -584,38 +600,46 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CP Marinade</t>
+          <t>star burger</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CP Marinade</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Crispy Chicken Patty</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>pc</t>
@@ -627,27 +651,31 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chicken 65</t>
+          <t>Hot Crispy burger</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chicken 65</t>
+          <t>Hot Crispy Patty</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -656,7 +684,11 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>pc</t>
@@ -670,29 +702,29 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Chicken Cheese Shotz</t>
+          <t>Paneer Delight burger</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Chicken Cheese Shotz</t>
+          <t>Paneer Patty</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -703,7 +735,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -726,22 +758,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chicken Fingers</t>
+          <t>Tandoori Burger Bun</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chicken Fingers</t>
+          <t>Tandoori Patty</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -750,7 +782,11 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>pc</t>
@@ -764,36 +800,40 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>95</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chicken Momos</t>
+          <t>Hungery bird burger</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Chicken Momos</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Whole Muscle Patty</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -807,34 +847,42 @@
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chicken Nuggets</t>
+          <t>Veg Burger</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chicken Nuggets</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>Veg Patty</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -850,29 +898,29 @@
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>65</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>BURGERS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chicken Popcorn</t>
+          <t>smokey burger</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chicken Popcorn</t>
+          <t>smokey burger</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -881,50 +929,54 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>129</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Chicken Strips</t>
+          <t>mirchi bites</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chicken Strips</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>mirchi bites</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -932,38 +984,38 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>109</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chilli Burst</t>
+          <t>saucy bites</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chilli Burst</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>boneless bites</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -977,44 +1029,40 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>99</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Crunchy Masala</t>
+          <t>chicken lollipops</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Crunchy Masala</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>chicken lollipops</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1022,127 +1070,135 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Eggless Mayonnaise</t>
+          <t>Mini Bucket</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eggless Mayonnaise</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>Thai Crispy</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>pc</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>385</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>French Fries</t>
+          <t>Big Buckets</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>French Fries</t>
+          <t>Thai Crispy</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>FRIED ITEM</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>765</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hot Crispy burger</t>
+          <t>Chicken Popcorn</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Hot Crispy Patty</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>Chicken Popcorn Small</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>pc</t>
+          <t>g</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1153,36 +1209,40 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>70</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hungery bird burger</t>
+          <t>Chicken Strips</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Whole Muscle Patty</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Chicken Strips</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1198,29 +1258,29 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>99</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Krusty Bites</t>
+          <t>Chilli Burst</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Krusty Bites</t>
+          <t>Chilli Burst</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>FRIED ITEM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1229,7 +1289,11 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1243,30 +1307,34 @@
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mini Bucket</t>
+          <t>Crunchy Masala</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
+          <t>Crunchy Masala</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1284,38 +1352,38 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>50</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Paneer Delight burger</t>
+          <t>Krusty Bites</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Paneer Patty</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>Krusty Bites</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1336,31 +1404,31 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rolls</t>
+          <t>FRIED ITEMS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Panner roll</t>
+          <t>Peri Peri Chwings</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>panner patty</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>Peri Peri Chwings</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1374,30 +1442,42 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>99</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>FRIED ITEMS</t>
+        </is>
+      </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Paratha</t>
+          <t>Thai Crispy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Paratha</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>Thai Crispy</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FRIED ITEM</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1409,32 +1489,44 @@
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>ROLLS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Paratha Sauce</t>
+          <t>Tandoori roll</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Paratha Sauce</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>chicken 65</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1446,27 +1538,31 @@
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>ROLLS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Peri Peri Chwings</t>
+          <t>Panner roll</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Peri Peri Chwings</t>
+          <t>panner patty</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>COMBO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1475,7 +1571,11 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1489,38 +1589,38 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>ROLLS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Pizza Pocket</t>
+          <t>Chicken Roll</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Pizza Pocket</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>chicken roll</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1532,40 +1632,36 @@
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>ROLLS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tandoori Burger Bun</t>
+          <t>KRISPER Roll</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tandoori Patty</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
+          <t>Krisper Roll</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1577,29 +1673,29 @@
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tandoori Mayonnaise</t>
+          <t>Paratha Sauce</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tandoori Mayonnaise</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>Paratha Sauce</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>1</t>
@@ -1623,22 +1719,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
+          <t>Tandoori Mayonnaise</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
+          <t>Tandoori Mayonnaise</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>SAUCE/DRY STOCK</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1647,11 +1743,7 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1663,40 +1755,36 @@
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Veg Burger</t>
+          <t>BBQ Seasoning</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Veg Patty</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>BBQ Seasoning</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1708,40 +1796,36 @@
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Veg Finger</t>
+          <t>CP Marinade</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Veg Finger</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>CP Marinade</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1753,40 +1837,36 @@
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rolls</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>chicken 65</t>
+          <t>Eggless Mayonnaise</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tandoori roll</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>Eggless Mayonnaise</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1798,206 +1878,250 @@
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
-      </c>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>chicken lollipops</t>
+          <t>PACKING COVER</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>chicken lollipops</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+          <t>PACKING COVER</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>pc</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>119</t>
-        </is>
-      </c>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>chicken popcorn large</t>
+          <t>SNACK BOX</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Chicken Popcorn</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>SNACK BOX</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>gms</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>cool drinks glass</t>
+          <t>French Fries</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>cool drinks</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>French Fries Small</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>50</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>masala fries Large</t>
+          <t>CHICKEN STRIPS</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>French Fries</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>CHICKEN STRIPS</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>COMBO</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>gms</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>85</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>snacks</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>mirchi bites</t>
+          <t>Chicken 65</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>mirchi bites</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>Chicken 65</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>85</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>pepsi 300 ml</t>
+          <t>Chicken Cheese Shotz</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>pepsi</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>Chicken Cheese Shotz</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>1</t>
@@ -2006,7 +2130,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>50</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2014,40 +2138,48 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Fried Items</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>saucy bites</t>
+          <t>Chicken Fingers</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>boneless bites</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>39</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2055,40 +2187,48 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>60</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>smokey burger</t>
+          <t>Chicken Momos</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>smokey burger</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>Chicken Momos</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2096,40 +2236,44 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>129</t>
-        </is>
-      </c>
+      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>star burger</t>
+          <t>Chicken Nuggets</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Crispy Chicken Patty</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>Chicken Nuggets</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2145,32 +2289,40 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>55</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>water 1/2 liter</t>
+          <t>Pizza Pocket</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>water</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>Pizza Pocket</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2178,13 +2330,246 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
+          <t>59</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Veg Finger</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Veg Finger</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>chicken popcorn large</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Chicken Popcorn Large</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>masala fries Large</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>French Fries Large</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>SNACKS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Burger Bun With Sesame</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Bun</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Paratha</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Paratha</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>STOCK</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>